<commit_message>
feat: complete v1.01 update for TBEA Dual-Center platform including indicator system v1.4, green power cards, dynamic tree, and dev docs
</commit_message>
<xml_diff>
--- a/需求文档/“双中心”数据需求清单V1.0/“双中心”项目能碳管控指标体系V1.4.xlsx
+++ b/需求文档/“双中心”数据需求清单V1.0/“双中心”项目能碳管控指标体系V1.4.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xwechat_files\wxid_uduybmyoqdj022_e7fe\msg\file\2026-08\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\TJ-nengtan\需求文档\“双中心”数据需求清单V1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="12080" tabRatio="319"/>
+    <workbookView windowWidth="28800" windowHeight="12255" tabRatio="319"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -5850,15 +5850,21 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <vertAlign val="subscript"/>
       <sz val="10.5"/>
       <name val="宋体"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="8"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
@@ -5872,12 +5878,6 @@
       <sz val="10.5"/>
       <color rgb="FFFF0000"/>
       <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <charset val="134"/>
     </font>
   </fonts>
@@ -6490,7 +6490,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -6581,11 +6581,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6733,7 +6742,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6021070" y="8467725"/>
+              <a:off x="6525895" y="8467725"/>
               <a:ext cx="405765" cy="393700"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -6774,7 +6783,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5890260" y="9879330"/>
+              <a:off x="6395085" y="9879330"/>
               <a:ext cx="850900" cy="393700"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -6815,7 +6824,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5872480" y="11045825"/>
+              <a:off x="6377305" y="11045825"/>
               <a:ext cx="1028700" cy="419100"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -6856,7 +6865,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6097905" y="12085320"/>
+              <a:off x="6602730" y="12085320"/>
               <a:ext cx="723900" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -6897,7 +6906,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5989955" y="13576300"/>
+              <a:off x="6494780" y="13576300"/>
               <a:ext cx="965200" cy="431800"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -6938,7 +6947,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6015355" y="2218690"/>
+              <a:off x="6520180" y="2218690"/>
               <a:ext cx="1117600" cy="419100"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -6979,7 +6988,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5873750" y="3388995"/>
+              <a:off x="6378575" y="3388995"/>
               <a:ext cx="1079500" cy="292100"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7020,7 +7029,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5605145" y="6129020"/>
+              <a:off x="6109970" y="6129020"/>
               <a:ext cx="1809750" cy="126365"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7061,7 +7070,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6259195" y="17231995"/>
+              <a:off x="6764020" y="17231995"/>
               <a:ext cx="419100" cy="393700"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7102,7 +7111,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6179820" y="19201765"/>
+              <a:off x="6684645" y="19201765"/>
               <a:ext cx="444500" cy="393700"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7143,7 +7152,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6073775" y="20440650"/>
+              <a:off x="6578600" y="20440650"/>
               <a:ext cx="596900" cy="405765"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7184,7 +7193,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5944870" y="21431885"/>
+              <a:off x="6449695" y="21431885"/>
               <a:ext cx="787400" cy="405765"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7225,7 +7234,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5911850" y="22148800"/>
+              <a:off x="6416675" y="22110700"/>
               <a:ext cx="965200" cy="405765"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7266,7 +7275,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6103620" y="23285450"/>
+              <a:off x="6608445" y="23247350"/>
               <a:ext cx="609600" cy="405765"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7307,7 +7316,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5767705" y="15654020"/>
+          <a:off x="6272530" y="15654020"/>
           <a:ext cx="1481455" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7349,7 +7358,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5752465" y="24825325"/>
+              <a:off x="6257290" y="24787225"/>
               <a:ext cx="1562100" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7390,7 +7399,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5704205" y="29913580"/>
+              <a:off x="6209030" y="29875480"/>
               <a:ext cx="1548765" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7431,7 +7440,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5619750" y="34418270"/>
+              <a:off x="6124575" y="34380170"/>
               <a:ext cx="1816100" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7472,7 +7481,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5622925" y="39283640"/>
+              <a:off x="6127750" y="39245540"/>
               <a:ext cx="1749425" cy="396240"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7513,7 +7522,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5674995" y="40860980"/>
+              <a:off x="6179820" y="40822880"/>
               <a:ext cx="1587500" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7554,7 +7563,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5596890" y="45712380"/>
+              <a:off x="6101715" y="45674280"/>
               <a:ext cx="1816100" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7595,7 +7604,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5602605" y="50697765"/>
+              <a:off x="6107430" y="50659665"/>
               <a:ext cx="1755775" cy="400050"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7636,7 +7645,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5843905" y="51932205"/>
+              <a:off x="6348730" y="51894105"/>
               <a:ext cx="1358900" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7677,7 +7686,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5799455" y="52955825"/>
+              <a:off x="6304280" y="52917725"/>
               <a:ext cx="1358900" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7718,7 +7727,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5737225" y="54154705"/>
+              <a:off x="6242050" y="54116605"/>
               <a:ext cx="1358900" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7759,7 +7768,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5749925" y="55693945"/>
+              <a:off x="6254750" y="55655845"/>
               <a:ext cx="1346200" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7800,7 +7809,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5777865" y="56938545"/>
+              <a:off x="6282690" y="56900445"/>
               <a:ext cx="1358900" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7841,7 +7850,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5786120" y="59034680"/>
+              <a:off x="6290945" y="58996580"/>
               <a:ext cx="1358900" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7882,7 +7891,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5691505" y="61066045"/>
+              <a:off x="6196330" y="61027945"/>
               <a:ext cx="1358900" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7923,7 +7932,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5727065" y="62122685"/>
+              <a:off x="6231890" y="62084585"/>
               <a:ext cx="1524000" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -7964,7 +7973,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5739765" y="63405385"/>
+              <a:off x="6244590" y="63367285"/>
               <a:ext cx="1524000" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8005,7 +8014,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5661025" y="64614425"/>
+              <a:off x="6165850" y="64576325"/>
               <a:ext cx="1714500" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8046,7 +8055,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5755005" y="65935225"/>
+              <a:off x="6259830" y="65897125"/>
               <a:ext cx="1346200" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8087,7 +8096,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5807075" y="67375405"/>
+              <a:off x="6311900" y="67337305"/>
               <a:ext cx="1346200" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8128,7 +8137,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5721985" y="68655565"/>
+              <a:off x="6226810" y="68617465"/>
               <a:ext cx="1346200" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8169,7 +8178,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5764530" y="69859525"/>
+              <a:off x="6269355" y="69821425"/>
               <a:ext cx="1358900" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8210,7 +8219,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5772785" y="71040625"/>
+              <a:off x="6277610" y="71002525"/>
               <a:ext cx="1346200" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8251,7 +8260,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5772785" y="71086345"/>
+              <a:off x="6277610" y="71048245"/>
               <a:ext cx="1346200" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8292,7 +8301,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5755005" y="72315705"/>
+              <a:off x="6259830" y="72277605"/>
               <a:ext cx="1358900" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8333,7 +8342,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5761355" y="74689970"/>
+              <a:off x="6266180" y="74651870"/>
               <a:ext cx="1459865" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8374,7 +8383,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5684520" y="75838685"/>
+              <a:off x="6189345" y="75800585"/>
               <a:ext cx="1459865" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8415,7 +8424,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5734685" y="77103605"/>
+              <a:off x="6239510" y="77065505"/>
               <a:ext cx="1459865" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8456,7 +8465,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5706745" y="78305025"/>
+              <a:off x="6211570" y="78266925"/>
               <a:ext cx="1473200" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8481,8 +8490,8 @@
         <xdr:to>
           <xdr:col>4</xdr:col>
           <xdr:colOff>1662430</xdr:colOff>
-          <xdr:row>64</xdr:row>
-          <xdr:rowOff>1008380</xdr:rowOff>
+          <xdr:row>65</xdr:row>
+          <xdr:rowOff>103505</xdr:rowOff>
         </xdr:to>
         <xdr:sp>
           <xdr:nvSpPr>
@@ -8497,7 +8506,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5742305" y="79681705"/>
+              <a:off x="6247130" y="79643605"/>
               <a:ext cx="1473200" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8538,7 +8547,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5755005" y="80683100"/>
+              <a:off x="6259830" y="80416400"/>
               <a:ext cx="1459865" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8579,7 +8588,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5754370" y="81968340"/>
+              <a:off x="6259195" y="81701640"/>
               <a:ext cx="1524000" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8620,7 +8629,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5683250" y="83337400"/>
+              <a:off x="6188075" y="83070700"/>
               <a:ext cx="1524000" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8661,7 +8670,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5574030" y="84620100"/>
+              <a:off x="6078855" y="84353400"/>
               <a:ext cx="1866900" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8702,7 +8711,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5557520" y="86102825"/>
+              <a:off x="6062345" y="85836125"/>
               <a:ext cx="1879600" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8743,7 +8752,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5742305" y="25805765"/>
+              <a:off x="6247130" y="25767665"/>
               <a:ext cx="1498600" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8784,7 +8793,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5634355" y="27256105"/>
+              <a:off x="6139180" y="27218005"/>
               <a:ext cx="1696720" cy="394335"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8825,7 +8834,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5880735" y="57970420"/>
+              <a:off x="6385560" y="57932320"/>
               <a:ext cx="1091565" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8866,7 +8875,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5682615" y="60009405"/>
+              <a:off x="6187440" y="59971305"/>
               <a:ext cx="1548765" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8907,7 +8916,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5662930" y="28634690"/>
+              <a:off x="6167755" y="28596590"/>
               <a:ext cx="1554480" cy="394335"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8948,7 +8957,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5670550" y="31395035"/>
+              <a:off x="6175375" y="31356935"/>
               <a:ext cx="1709420" cy="358140"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -8989,7 +8998,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5645150" y="32898715"/>
+              <a:off x="6149975" y="32860615"/>
               <a:ext cx="1699895" cy="358140"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -9030,7 +9039,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5603240" y="36095305"/>
+              <a:off x="6108065" y="36057205"/>
               <a:ext cx="1830070" cy="341630"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -9071,7 +9080,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5578475" y="37754560"/>
+              <a:off x="6083300" y="37716460"/>
               <a:ext cx="1821180" cy="341630"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -9112,7 +9121,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5641975" y="42548175"/>
+              <a:off x="6146800" y="42510075"/>
               <a:ext cx="1730375" cy="358140"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -9153,7 +9162,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5581015" y="44222670"/>
+              <a:off x="6085840" y="44184570"/>
               <a:ext cx="1816735" cy="387985"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -9194,7 +9203,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5603240" y="47385605"/>
+              <a:off x="6108065" y="47347505"/>
               <a:ext cx="1830070" cy="341630"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -9235,7 +9244,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5578475" y="49044860"/>
+              <a:off x="6083300" y="49006760"/>
               <a:ext cx="1821180" cy="341630"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -9276,7 +9285,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5583555" y="73595230"/>
+              <a:off x="6088380" y="73557130"/>
               <a:ext cx="1816100" cy="457200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -9543,22 +9552,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:Y86"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="5.81818181818182" customWidth="1"/>
-    <col min="2" max="2" width="16.4636363636364" customWidth="1"/>
-    <col min="3" max="3" width="29.4181818181818" customWidth="1"/>
+    <col min="1" max="1" width="5.81666666666667" customWidth="1"/>
+    <col min="2" max="2" width="16.4666666666667" customWidth="1"/>
+    <col min="3" max="3" width="29.4166666666667" customWidth="1"/>
     <col min="4" max="4" width="27.8" customWidth="1"/>
-    <col min="5" max="5" width="27.5909090909091" customWidth="1"/>
-    <col min="6" max="6" width="53.5909090909091" style="2" customWidth="1"/>
-    <col min="7" max="7" width="25.1818181818182" customWidth="1"/>
-    <col min="8" max="8" width="11.8818181818182" customWidth="1"/>
-    <col min="9" max="9" width="10.4909090909091" customWidth="1"/>
+    <col min="5" max="5" width="27.5916666666667" customWidth="1"/>
+    <col min="6" max="6" width="53.5916666666667" style="2" customWidth="1"/>
+    <col min="7" max="7" width="25.1833333333333" customWidth="1"/>
+    <col min="8" max="8" width="11.8833333333333" customWidth="1"/>
+    <col min="9" max="9" width="10.4916666666667" customWidth="1"/>
     <col min="10" max="10" width="15.2" customWidth="1"/>
-    <col min="11" max="11" width="14.9181818181818" customWidth="1"/>
-    <col min="12" max="12" width="40.2545454545455" style="2" customWidth="1"/>
-    <col min="13" max="13" width="58.1818181818182" style="2" customWidth="1"/>
-    <col min="14" max="14" width="41.5545454545455" customWidth="1"/>
+    <col min="11" max="11" width="14.9166666666667" customWidth="1"/>
+    <col min="12" max="12" width="40.2583333333333" style="2" customWidth="1"/>
+    <col min="13" max="13" width="58.1833333333333" style="2" customWidth="1"/>
+    <col min="14" max="14" width="41.5583333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:25">
@@ -10165,7 +10174,7 @@
       </c>
       <c r="M17" s="26"/>
     </row>
-    <row r="18" ht="54.75" spans="1:15">
+    <row r="18" ht="51.75" spans="1:15">
       <c r="A18" s="20">
         <v>14</v>
       </c>
@@ -10317,13 +10326,13 @@
       <c r="J22" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K22" s="24" t="s">
+      <c r="K22" s="30" t="s">
         <v>117</v>
       </c>
       <c r="L22" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="M22" s="30" t="s">
+      <c r="M22" s="31" t="s">
         <v>119</v>
       </c>
     </row>
@@ -10354,11 +10363,11 @@
       <c r="J23" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K23" s="24"/>
+      <c r="K23" s="32"/>
       <c r="L23" s="26" t="s">
         <v>123</v>
       </c>
-      <c r="M23" s="30" t="s">
+      <c r="M23" s="31" t="s">
         <v>124</v>
       </c>
     </row>
@@ -10389,11 +10398,11 @@
       <c r="J24" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K24" s="24"/>
+      <c r="K24" s="32"/>
       <c r="L24" s="26" t="s">
         <v>129</v>
       </c>
-      <c r="M24" s="31" t="s">
+      <c r="M24" s="33" t="s">
         <v>130</v>
       </c>
       <c r="N24" s="28" t="s">
@@ -10427,15 +10436,15 @@
       <c r="J25" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K25" s="24"/>
+      <c r="K25" s="34"/>
       <c r="L25" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="M25" s="31" t="s">
+      <c r="M25" s="33" t="s">
         <v>136</v>
       </c>
-      <c r="N25" s="32"/>
-      <c r="O25" s="32"/>
+      <c r="N25" s="35"/>
+      <c r="O25" s="35"/>
     </row>
     <row r="26" s="1" customFormat="1" ht="112" customHeight="1" spans="1:15">
       <c r="A26" s="25"/>
@@ -10470,13 +10479,13 @@
       <c r="L26" s="26" t="s">
         <v>142</v>
       </c>
-      <c r="M26" s="31" t="s">
+      <c r="M26" s="33" t="s">
         <v>143</v>
       </c>
-      <c r="N26" s="32" t="s">
+      <c r="N26" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="O26" s="32"/>
+      <c r="O26" s="35"/>
     </row>
     <row r="27" s="1" customFormat="1" ht="112" customHeight="1" spans="1:15">
       <c r="A27" s="25"/>
@@ -10507,9 +10516,9 @@
       </c>
       <c r="K27" s="24"/>
       <c r="L27" s="26"/>
-      <c r="M27" s="31"/>
-      <c r="N27" s="32"/>
-      <c r="O27" s="32"/>
+      <c r="M27" s="33"/>
+      <c r="N27" s="35"/>
+      <c r="O27" s="35"/>
     </row>
     <row r="28" s="1" customFormat="1" ht="119" customHeight="1" spans="1:15">
       <c r="A28" s="25"/>
@@ -10540,9 +10549,9 @@
       </c>
       <c r="K28" s="24"/>
       <c r="L28" s="26"/>
-      <c r="M28" s="31"/>
-      <c r="N28" s="32"/>
-      <c r="O28" s="32"/>
+      <c r="M28" s="33"/>
+      <c r="N28" s="35"/>
+      <c r="O28" s="35"/>
     </row>
     <row r="29" s="1" customFormat="1" ht="127" customHeight="1" spans="1:15">
       <c r="A29" s="25"/>
@@ -10573,11 +10582,11 @@
       </c>
       <c r="K29" s="24"/>
       <c r="L29" s="26"/>
-      <c r="M29" s="31"/>
-      <c r="N29" s="32" t="s">
+      <c r="M29" s="33"/>
+      <c r="N29" s="35" t="s">
         <v>155</v>
       </c>
-      <c r="O29" s="32"/>
+      <c r="O29" s="35"/>
     </row>
     <row r="30" s="1" customFormat="1" ht="127" customHeight="1" spans="1:15">
       <c r="A30" s="25"/>
@@ -10608,9 +10617,9 @@
       </c>
       <c r="K30" s="24"/>
       <c r="L30" s="26"/>
-      <c r="M30" s="31"/>
-      <c r="N30" s="32"/>
-      <c r="O30" s="32"/>
+      <c r="M30" s="33"/>
+      <c r="N30" s="35"/>
+      <c r="O30" s="35"/>
     </row>
     <row r="31" s="1" customFormat="1" ht="127" customHeight="1" spans="1:15">
       <c r="A31" s="25"/>
@@ -10641,9 +10650,9 @@
       </c>
       <c r="K31" s="24"/>
       <c r="L31" s="26"/>
-      <c r="M31" s="31"/>
-      <c r="N31" s="32"/>
-      <c r="O31" s="32"/>
+      <c r="M31" s="33"/>
+      <c r="N31" s="35"/>
+      <c r="O31" s="35"/>
     </row>
     <row r="32" s="1" customFormat="1" ht="127" customHeight="1" spans="1:15">
       <c r="A32" s="25"/>
@@ -10674,9 +10683,9 @@
       </c>
       <c r="K32" s="24"/>
       <c r="L32" s="26"/>
-      <c r="M32" s="31"/>
-      <c r="N32" s="32"/>
-      <c r="O32" s="32"/>
+      <c r="M32" s="33"/>
+      <c r="N32" s="35"/>
+      <c r="O32" s="35"/>
     </row>
     <row r="33" s="1" customFormat="1" ht="127" customHeight="1" spans="1:15">
       <c r="A33" s="25"/>
@@ -10709,11 +10718,11 @@
       <c r="L33" s="26" t="s">
         <v>170</v>
       </c>
-      <c r="M33" s="31" t="s">
+      <c r="M33" s="33" t="s">
         <v>171</v>
       </c>
-      <c r="N33" s="32"/>
-      <c r="O33" s="32"/>
+      <c r="N33" s="35"/>
+      <c r="O33" s="35"/>
     </row>
     <row r="34" s="1" customFormat="1" ht="127" customHeight="1" spans="1:15">
       <c r="A34" s="25"/>
@@ -10744,9 +10753,9 @@
       </c>
       <c r="K34" s="24"/>
       <c r="L34" s="26"/>
-      <c r="M34" s="31"/>
-      <c r="N34" s="32"/>
-      <c r="O34" s="32"/>
+      <c r="M34" s="33"/>
+      <c r="N34" s="35"/>
+      <c r="O34" s="35"/>
     </row>
     <row r="35" s="1" customFormat="1" ht="127" customHeight="1" spans="1:15">
       <c r="A35" s="25"/>
@@ -10777,9 +10786,9 @@
       </c>
       <c r="K35" s="24"/>
       <c r="L35" s="26"/>
-      <c r="M35" s="31"/>
-      <c r="N35" s="32"/>
-      <c r="O35" s="32"/>
+      <c r="M35" s="33"/>
+      <c r="N35" s="35"/>
+      <c r="O35" s="35"/>
     </row>
     <row r="36" s="1" customFormat="1" ht="127" customHeight="1" spans="1:15">
       <c r="A36" s="25"/>
@@ -10810,9 +10819,9 @@
       </c>
       <c r="K36" s="24"/>
       <c r="L36" s="26"/>
-      <c r="M36" s="31"/>
-      <c r="N36" s="32"/>
-      <c r="O36" s="32"/>
+      <c r="M36" s="33"/>
+      <c r="N36" s="35"/>
+      <c r="O36" s="35"/>
     </row>
     <row r="37" s="1" customFormat="1" ht="127" customHeight="1" spans="1:15">
       <c r="A37" s="25"/>
@@ -10843,9 +10852,9 @@
       </c>
       <c r="K37" s="24"/>
       <c r="L37" s="26"/>
-      <c r="M37" s="31"/>
-      <c r="N37" s="32"/>
-      <c r="O37" s="32"/>
+      <c r="M37" s="33"/>
+      <c r="N37" s="35"/>
+      <c r="O37" s="35"/>
     </row>
     <row r="38" s="1" customFormat="1" ht="127" customHeight="1" spans="1:15">
       <c r="A38" s="25"/>
@@ -10876,9 +10885,9 @@
       </c>
       <c r="K38" s="24"/>
       <c r="L38" s="26"/>
-      <c r="M38" s="31"/>
-      <c r="N38" s="32"/>
-      <c r="O38" s="32"/>
+      <c r="M38" s="33"/>
+      <c r="N38" s="35"/>
+      <c r="O38" s="35"/>
     </row>
     <row r="39" s="1" customFormat="1" ht="127" customHeight="1" spans="1:15">
       <c r="A39" s="25"/>
@@ -10909,9 +10918,9 @@
       </c>
       <c r="K39" s="24"/>
       <c r="L39" s="26"/>
-      <c r="M39" s="31"/>
-      <c r="N39" s="32"/>
-      <c r="O39" s="32"/>
+      <c r="M39" s="33"/>
+      <c r="N39" s="35"/>
+      <c r="O39" s="35"/>
     </row>
     <row r="40" s="1" customFormat="1" ht="85" customHeight="1" spans="1:15">
       <c r="A40" s="25"/>
@@ -10944,11 +10953,11 @@
       <c r="L40" s="26" t="s">
         <v>193</v>
       </c>
-      <c r="M40" s="33" t="s">
+      <c r="M40" s="36" t="s">
         <v>194</v>
       </c>
-      <c r="N40" s="32"/>
-      <c r="O40" s="32"/>
+      <c r="N40" s="35"/>
+      <c r="O40" s="35"/>
     </row>
     <row r="41" s="1" customFormat="1" ht="81" customHeight="1" spans="1:15">
       <c r="A41" s="25"/>
@@ -10981,11 +10990,11 @@
       <c r="L41" s="26" t="s">
         <v>198</v>
       </c>
-      <c r="M41" s="33" t="s">
+      <c r="M41" s="36" t="s">
         <v>199</v>
       </c>
-      <c r="N41" s="32"/>
-      <c r="O41" s="32"/>
+      <c r="N41" s="35"/>
+      <c r="O41" s="35"/>
     </row>
     <row r="42" s="1" customFormat="1" ht="116" customHeight="1" spans="1:15">
       <c r="A42" s="25"/>
@@ -10995,7 +11004,7 @@
       <c r="C42" s="24" t="s">
         <v>200</v>
       </c>
-      <c r="D42" s="34" t="s">
+      <c r="D42" s="37" t="s">
         <v>201</v>
       </c>
       <c r="E42" s="24"/>
@@ -11020,7 +11029,7 @@
       <c r="L42" s="26" t="s">
         <v>204</v>
       </c>
-      <c r="M42" s="33" t="s">
+      <c r="M42" s="36" t="s">
         <v>205</v>
       </c>
       <c r="N42" s="1" t="s">
@@ -11035,7 +11044,7 @@
       <c r="C43" s="24" t="s">
         <v>207</v>
       </c>
-      <c r="D43" s="34" t="s">
+      <c r="D43" s="37" t="s">
         <v>208</v>
       </c>
       <c r="E43" s="24"/>
@@ -11060,7 +11069,7 @@
       <c r="L43" s="26" t="s">
         <v>210</v>
       </c>
-      <c r="M43" s="33" t="s">
+      <c r="M43" s="36" t="s">
         <v>211</v>
       </c>
     </row>
@@ -11091,13 +11100,13 @@
       <c r="J44" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K44" s="35" t="s">
+      <c r="K44" s="38" t="s">
         <v>215</v>
       </c>
       <c r="L44" s="26" t="s">
         <v>216</v>
       </c>
-      <c r="M44" s="33" t="s">
+      <c r="M44" s="36" t="s">
         <v>217</v>
       </c>
       <c r="N44" s="1" t="s">
@@ -11112,7 +11121,7 @@
       <c r="C45" s="24" t="s">
         <v>219</v>
       </c>
-      <c r="D45" s="34" t="s">
+      <c r="D45" s="37" t="s">
         <v>220</v>
       </c>
       <c r="E45" s="24"/>
@@ -11131,11 +11140,11 @@
       <c r="J45" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K45" s="36"/>
+      <c r="K45" s="39"/>
       <c r="L45" s="26" t="s">
         <v>222</v>
       </c>
-      <c r="M45" s="33" t="s">
+      <c r="M45" s="36" t="s">
         <v>223</v>
       </c>
     </row>
@@ -11147,7 +11156,7 @@
       <c r="C46" s="24" t="s">
         <v>224</v>
       </c>
-      <c r="D46" s="34" t="s">
+      <c r="D46" s="37" t="s">
         <v>225</v>
       </c>
       <c r="E46" s="24"/>
@@ -11166,11 +11175,11 @@
       <c r="J46" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K46" s="37"/>
+      <c r="K46" s="40"/>
       <c r="L46" s="26" t="s">
         <v>227</v>
       </c>
-      <c r="M46" s="33" t="s">
+      <c r="M46" s="36" t="s">
         <v>228</v>
       </c>
     </row>
@@ -11182,7 +11191,7 @@
       <c r="C47" s="24" t="s">
         <v>229</v>
       </c>
-      <c r="D47" s="34" t="s">
+      <c r="D47" s="37" t="s">
         <v>230</v>
       </c>
       <c r="E47" s="24"/>
@@ -11201,13 +11210,13 @@
       <c r="J47" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K47" s="35" t="s">
+      <c r="K47" s="38" t="s">
         <v>232</v>
       </c>
       <c r="L47" s="26" t="s">
         <v>233</v>
       </c>
-      <c r="M47" s="38" t="s">
+      <c r="M47" s="41" t="s">
         <v>234</v>
       </c>
       <c r="N47" s="1" t="s">
@@ -11241,11 +11250,11 @@
       <c r="J48" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K48" s="36"/>
+      <c r="K48" s="39"/>
       <c r="L48" s="26" t="s">
         <v>238</v>
       </c>
-      <c r="M48" s="39"/>
+      <c r="M48" s="42"/>
     </row>
     <row r="49" s="1" customFormat="1" ht="81" customHeight="1" spans="1:14">
       <c r="A49" s="25"/>
@@ -11274,11 +11283,11 @@
       <c r="J49" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K49" s="36"/>
+      <c r="K49" s="39"/>
       <c r="L49" s="26" t="s">
         <v>242</v>
       </c>
-      <c r="M49" s="40"/>
+      <c r="M49" s="43"/>
     </row>
     <row r="50" s="1" customFormat="1" ht="81" customHeight="1" spans="1:14">
       <c r="A50" s="25"/>
@@ -11288,7 +11297,7 @@
       <c r="C50" s="24" t="s">
         <v>243</v>
       </c>
-      <c r="D50" s="34" t="s">
+      <c r="D50" s="37" t="s">
         <v>244</v>
       </c>
       <c r="E50" s="24"/>
@@ -11307,11 +11316,11 @@
       <c r="J50" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K50" s="37"/>
+      <c r="K50" s="40"/>
       <c r="L50" s="26" t="s">
         <v>246</v>
       </c>
-      <c r="M50" s="33" t="s">
+      <c r="M50" s="36" t="s">
         <v>247</v>
       </c>
     </row>
@@ -11320,10 +11329,10 @@
       <c r="B51" s="21">
         <v>46</v>
       </c>
-      <c r="C51" s="41" t="s">
+      <c r="C51" s="44" t="s">
         <v>248</v>
       </c>
-      <c r="D51" s="34" t="s">
+      <c r="D51" s="37" t="s">
         <v>249</v>
       </c>
       <c r="E51" s="24"/>
@@ -11342,13 +11351,13 @@
       <c r="J51" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K51" s="42" t="s">
+      <c r="K51" s="45" t="s">
         <v>251</v>
       </c>
       <c r="L51" s="26" t="s">
         <v>252</v>
       </c>
-      <c r="M51" s="33" t="s">
+      <c r="M51" s="36" t="s">
         <v>253</v>
       </c>
     </row>
@@ -11357,10 +11366,10 @@
       <c r="B52" s="21">
         <v>47</v>
       </c>
-      <c r="C52" s="41" t="s">
+      <c r="C52" s="44" t="s">
         <v>254</v>
       </c>
-      <c r="D52" s="34" t="s">
+      <c r="D52" s="37" t="s">
         <v>255</v>
       </c>
       <c r="E52" s="24"/>
@@ -11379,11 +11388,11 @@
       <c r="J52" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K52" s="43"/>
+      <c r="K52" s="46"/>
       <c r="L52" s="26" t="s">
         <v>257</v>
       </c>
-      <c r="M52" s="33" t="s">
+      <c r="M52" s="36" t="s">
         <v>258</v>
       </c>
     </row>
@@ -11392,10 +11401,10 @@
       <c r="B53" s="21">
         <v>48</v>
       </c>
-      <c r="C53" s="41" t="s">
+      <c r="C53" s="44" t="s">
         <v>259</v>
       </c>
-      <c r="D53" s="34" t="s">
+      <c r="D53" s="37" t="s">
         <v>260</v>
       </c>
       <c r="E53" s="24"/>
@@ -11414,11 +11423,11 @@
       <c r="J53" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K53" s="44"/>
+      <c r="K53" s="47"/>
       <c r="L53" s="26" t="s">
         <v>262</v>
       </c>
-      <c r="M53" s="33" t="s">
+      <c r="M53" s="36" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11430,14 +11439,14 @@
       <c r="C54" s="24" t="s">
         <v>264</v>
       </c>
-      <c r="D54" s="34" t="s">
+      <c r="D54" s="37" t="s">
         <v>265</v>
       </c>
       <c r="E54" s="24"/>
-      <c r="F54" s="34" t="s">
+      <c r="F54" s="37" t="s">
         <v>266</v>
       </c>
-      <c r="G54" s="45" t="s">
+      <c r="G54" s="48" t="s">
         <v>267</v>
       </c>
       <c r="H54" s="24" t="s">
@@ -11449,13 +11458,13 @@
       <c r="J54" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K54" s="45" t="s">
+      <c r="K54" s="48" t="s">
         <v>268</v>
       </c>
       <c r="L54" s="26" t="s">
         <v>269</v>
       </c>
-      <c r="M54" s="33" t="s">
+      <c r="M54" s="36" t="s">
         <v>270</v>
       </c>
       <c r="N54" s="1" t="s">
@@ -11470,14 +11479,14 @@
       <c r="C55" s="24" t="s">
         <v>272</v>
       </c>
-      <c r="D55" s="34" t="s">
+      <c r="D55" s="37" t="s">
         <v>273</v>
       </c>
       <c r="E55" s="24"/>
-      <c r="F55" s="34" t="s">
+      <c r="F55" s="37" t="s">
         <v>274</v>
       </c>
-      <c r="G55" s="45" t="s">
+      <c r="G55" s="48" t="s">
         <v>267</v>
       </c>
       <c r="H55" s="24" t="s">
@@ -11489,11 +11498,11 @@
       <c r="J55" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K55" s="45"/>
+      <c r="K55" s="48"/>
       <c r="L55" s="26" t="s">
         <v>275</v>
       </c>
-      <c r="M55" s="33" t="s">
+      <c r="M55" s="36" t="s">
         <v>276</v>
       </c>
       <c r="N55" s="1" t="s">
@@ -11508,14 +11517,14 @@
       <c r="C56" s="24" t="s">
         <v>278</v>
       </c>
-      <c r="D56" s="34" t="s">
+      <c r="D56" s="37" t="s">
         <v>279</v>
       </c>
       <c r="E56" s="24"/>
-      <c r="F56" s="34" t="s">
+      <c r="F56" s="37" t="s">
         <v>280</v>
       </c>
-      <c r="G56" s="45" t="s">
+      <c r="G56" s="48" t="s">
         <v>267</v>
       </c>
       <c r="H56" s="24" t="s">
@@ -11527,11 +11536,11 @@
       <c r="J56" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K56" s="45"/>
+      <c r="K56" s="48"/>
       <c r="L56" s="26" t="s">
         <v>281</v>
       </c>
-      <c r="M56" s="33" t="s">
+      <c r="M56" s="36" t="s">
         <v>282</v>
       </c>
       <c r="N56" s="1" t="s">
@@ -11546,14 +11555,14 @@
       <c r="C57" s="24" t="s">
         <v>283</v>
       </c>
-      <c r="D57" s="34" t="s">
+      <c r="D57" s="37" t="s">
         <v>284</v>
       </c>
       <c r="E57" s="24"/>
-      <c r="F57" s="34" t="s">
+      <c r="F57" s="37" t="s">
         <v>285</v>
       </c>
-      <c r="G57" s="45" t="s">
+      <c r="G57" s="48" t="s">
         <v>267</v>
       </c>
       <c r="H57" s="24" t="s">
@@ -11565,11 +11574,11 @@
       <c r="J57" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K57" s="45"/>
+      <c r="K57" s="48"/>
       <c r="L57" s="26" t="s">
         <v>286</v>
       </c>
-      <c r="M57" s="33" t="s">
+      <c r="M57" s="36" t="s">
         <v>287</v>
       </c>
       <c r="N57" s="1" t="s">
@@ -11584,7 +11593,7 @@
       <c r="C58" s="24" t="s">
         <v>288</v>
       </c>
-      <c r="D58" s="34" t="s">
+      <c r="D58" s="37" t="s">
         <v>289</v>
       </c>
       <c r="E58" s="24"/>
@@ -11603,13 +11612,13 @@
       <c r="J58" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K58" s="45" t="s">
+      <c r="K58" s="48" t="s">
         <v>291</v>
       </c>
       <c r="L58" s="26" t="s">
         <v>292</v>
       </c>
-      <c r="M58" s="33" t="s">
+      <c r="M58" s="36" t="s">
         <v>293</v>
       </c>
       <c r="N58" s="1" t="s">
@@ -11624,7 +11633,7 @@
       <c r="C59" s="24" t="s">
         <v>295</v>
       </c>
-      <c r="D59" s="34" t="s">
+      <c r="D59" s="37" t="s">
         <v>296</v>
       </c>
       <c r="E59" s="24"/>
@@ -11643,11 +11652,11 @@
       <c r="J59" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K59" s="45"/>
+      <c r="K59" s="48"/>
       <c r="L59" s="26" t="s">
         <v>298</v>
       </c>
-      <c r="M59" s="33" t="s">
+      <c r="M59" s="36" t="s">
         <v>299</v>
       </c>
       <c r="N59" s="1" t="s">
@@ -11659,10 +11668,10 @@
       <c r="B60" s="21">
         <v>55</v>
       </c>
-      <c r="C60" s="46" t="s">
+      <c r="C60" s="49" t="s">
         <v>301</v>
       </c>
-      <c r="D60" s="47" t="s">
+      <c r="D60" s="50" t="s">
         <v>302</v>
       </c>
       <c r="E60" s="24"/>
@@ -11681,13 +11690,13 @@
       <c r="J60" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K60" s="43" t="s">
+      <c r="K60" s="46" t="s">
         <v>304</v>
       </c>
       <c r="L60" s="26" t="s">
         <v>305</v>
       </c>
-      <c r="M60" s="33" t="s">
+      <c r="M60" s="36" t="s">
         <v>306</v>
       </c>
       <c r="N60" s="1" t="s">
@@ -11702,7 +11711,7 @@
       <c r="C61" s="24" t="s">
         <v>307</v>
       </c>
-      <c r="D61" s="34" t="s">
+      <c r="D61" s="37" t="s">
         <v>308</v>
       </c>
       <c r="E61" s="24"/>
@@ -11721,11 +11730,11 @@
       <c r="J61" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K61" s="43"/>
+      <c r="K61" s="46"/>
       <c r="L61" s="26" t="s">
         <v>310</v>
       </c>
-      <c r="M61" s="33" t="s">
+      <c r="M61" s="36" t="s">
         <v>306</v>
       </c>
       <c r="N61" s="28"/>
@@ -11738,7 +11747,7 @@
       <c r="C62" s="24" t="s">
         <v>311</v>
       </c>
-      <c r="D62" s="34" t="s">
+      <c r="D62" s="37" t="s">
         <v>312</v>
       </c>
       <c r="E62" s="24"/>
@@ -11757,11 +11766,11 @@
       <c r="J62" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K62" s="43"/>
+      <c r="K62" s="46"/>
       <c r="L62" s="26" t="s">
         <v>314</v>
       </c>
-      <c r="M62" s="33" t="s">
+      <c r="M62" s="36" t="s">
         <v>315</v>
       </c>
     </row>
@@ -11773,7 +11782,7 @@
       <c r="C63" s="24" t="s">
         <v>316</v>
       </c>
-      <c r="D63" s="34" t="s">
+      <c r="D63" s="37" t="s">
         <v>317</v>
       </c>
       <c r="E63" s="24"/>
@@ -11792,13 +11801,13 @@
       <c r="J63" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K63" s="42" t="s">
+      <c r="K63" s="45" t="s">
         <v>319</v>
       </c>
       <c r="L63" s="26" t="s">
         <v>320</v>
       </c>
-      <c r="M63" s="33" t="s">
+      <c r="M63" s="36" t="s">
         <v>321</v>
       </c>
       <c r="N63" s="1" t="s">
@@ -11813,7 +11822,7 @@
       <c r="C64" s="24" t="s">
         <v>323</v>
       </c>
-      <c r="D64" s="34" t="s">
+      <c r="D64" s="37" t="s">
         <v>324</v>
       </c>
       <c r="E64" s="24"/>
@@ -11832,15 +11841,15 @@
       <c r="J64" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K64" s="43"/>
+      <c r="K64" s="46"/>
       <c r="L64" s="26" t="s">
         <v>326</v>
       </c>
-      <c r="M64" s="33" t="s">
+      <c r="M64" s="36" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="65" s="1" customFormat="1" ht="89.25" spans="1:13">
+    <row r="65" s="1" customFormat="1" ht="71.25" spans="1:13">
       <c r="A65" s="25"/>
       <c r="B65" s="21">
         <v>60</v>
@@ -11848,7 +11857,7 @@
       <c r="C65" s="24" t="s">
         <v>328</v>
       </c>
-      <c r="D65" s="34" t="s">
+      <c r="D65" s="37" t="s">
         <v>329</v>
       </c>
       <c r="E65" s="24"/>
@@ -11867,11 +11876,11 @@
       <c r="J65" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K65" s="43"/>
+      <c r="K65" s="46"/>
       <c r="L65" s="26" t="s">
         <v>331</v>
       </c>
-      <c r="M65" s="33" t="s">
+      <c r="M65" s="36" t="s">
         <v>332</v>
       </c>
     </row>
@@ -11883,7 +11892,7 @@
       <c r="C66" s="24" t="s">
         <v>333</v>
       </c>
-      <c r="D66" s="34" t="s">
+      <c r="D66" s="37" t="s">
         <v>334</v>
       </c>
       <c r="E66" s="24"/>
@@ -11902,11 +11911,11 @@
       <c r="J66" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K66" s="44"/>
+      <c r="K66" s="47"/>
       <c r="L66" s="26" t="s">
         <v>336</v>
       </c>
-      <c r="M66" s="33" t="s">
+      <c r="M66" s="36" t="s">
         <v>337</v>
       </c>
     </row>
@@ -11937,18 +11946,18 @@
       <c r="J67" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K67" s="42" t="s">
+      <c r="K67" s="45" t="s">
         <v>341</v>
       </c>
       <c r="L67" s="26" t="s">
         <v>342</v>
       </c>
-      <c r="M67" s="33" t="s">
+      <c r="M67" s="36" t="s">
         <v>343</v>
       </c>
     </row>
     <row r="68" s="1" customFormat="1" ht="106" customHeight="1" spans="1:13">
-      <c r="A68" s="48"/>
+      <c r="A68" s="51"/>
       <c r="B68" s="21">
         <v>63</v>
       </c>
@@ -11974,16 +11983,16 @@
       <c r="J68" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K68" s="43"/>
+      <c r="K68" s="46"/>
       <c r="L68" s="26" t="s">
         <v>347</v>
       </c>
-      <c r="M68" s="33" t="s">
+      <c r="M68" s="36" t="s">
         <v>348</v>
       </c>
     </row>
     <row r="69" s="1" customFormat="1" ht="112" customHeight="1" spans="1:13">
-      <c r="A69" s="49"/>
+      <c r="A69" s="52"/>
       <c r="B69" s="21">
         <v>64</v>
       </c>
@@ -12009,16 +12018,16 @@
       <c r="J69" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K69" s="43"/>
+      <c r="K69" s="46"/>
       <c r="L69" s="26" t="s">
         <v>352</v>
       </c>
-      <c r="M69" s="33" t="s">
+      <c r="M69" s="36" t="s">
         <v>353</v>
       </c>
     </row>
     <row r="70" s="1" customFormat="1" ht="112" customHeight="1" spans="1:13">
-      <c r="A70" s="49"/>
+      <c r="A70" s="52"/>
       <c r="B70" s="21">
         <v>65</v>
       </c>
@@ -12044,11 +12053,11 @@
       <c r="J70" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="K70" s="44"/>
+      <c r="K70" s="47"/>
       <c r="L70" s="26" t="s">
         <v>357</v>
       </c>
-      <c r="M70" s="33" t="s">
+      <c r="M70" s="36" t="s">
         <v>358</v>
       </c>
     </row>
@@ -12076,7 +12085,7 @@
     <mergeCell ref="B21:M21"/>
     <mergeCell ref="K4:K14"/>
     <mergeCell ref="K16:K20"/>
-    <mergeCell ref="K22:K24"/>
+    <mergeCell ref="K22:K25"/>
     <mergeCell ref="K26:K41"/>
     <mergeCell ref="K44:K46"/>
     <mergeCell ref="K47:K50"/>
@@ -13164,8 +13173,8 @@
               <to>
                 <xdr:col>4</xdr:col>
                 <xdr:colOff>1662430</xdr:colOff>
-                <xdr:row>64</xdr:row>
-                <xdr:rowOff>1008380</xdr:rowOff>
+                <xdr:row>65</xdr:row>
+                <xdr:rowOff>103505</xdr:rowOff>
               </to>
             </anchor>
           </objectPr>
@@ -13658,7 +13667,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -13670,7 +13679,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>